<commit_message>
B14 e B8 fecham: o TR treinado soma a maestria (limpeza 9 da ficha-v01, catalogo em maestria, regressao da Kaori nos quatro TRs); a nota da CD e o conferir-kaori saem da regra velha, o conferir-kaori passa a falhar de verdade, e a Integridade do catalogo vai para a formula do manual; a sub_origem e as rotas_de_criacao do catalogo passam a seguir o livro e saem das nao conferidas; o catalogo e o carimbo vao a v0.240; o B19 e escrito no Codigo.gs, falta testar no Sheets
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ficha-v01/ficha-projeto-m-0.1.xlsx
+++ b/ficha-v01/ficha-projeto-m-0.1.xlsx
@@ -8015,7 +8015,7 @@
       <c r="AN75" s="10" t="n"/>
       <c r="AO75" s="11" t="n"/>
       <c r="AP75" s="95">
-        <f>+IFS(AK75="FORÇA",$D$17, AK75="DESTREZA",$L$17)+IF($AF$75=TRUE,2,0)+AJ75</f>
+        <f>+IFS(AK75="FORÇA",$D$17, AK75="DESTREZA",$L$17)+IF($AF$75=TRUE,$D$48,0)+AJ75</f>
         <v/>
       </c>
       <c r="AQ75" s="10" t="n"/>
@@ -8106,7 +8106,7 @@
       <c r="AN76" s="10" t="n"/>
       <c r="AO76" s="11" t="n"/>
       <c r="AP76" s="95">
-        <f>$T$17+IF($AF$76=TRUE,2,0)+AJ76</f>
+        <f>$T$17+IF($AF$76=TRUE,$D$48,0)+AJ76</f>
         <v/>
       </c>
       <c r="AQ76" s="10" t="n"/>
@@ -8197,7 +8197,7 @@
       <c r="AN77" s="10" t="n"/>
       <c r="AO77" s="11" t="n"/>
       <c r="AP77" s="95">
-        <f>$AB$17+IF($AF$77=TRUE,2,0)+AJ77</f>
+        <f>$AB$17+IF($AF$77=TRUE,$D$48,0)+AJ77</f>
         <v/>
       </c>
       <c r="AQ77" s="10" t="n"/>
@@ -8288,7 +8288,7 @@
       <c r="AN78" s="10" t="n"/>
       <c r="AO78" s="11" t="n"/>
       <c r="AP78" s="95">
-        <f>$AJ$17+IF($AF$78=TRUE,2,0)+AJ78</f>
+        <f>$AJ$17+IF($AF$78=TRUE,$D$48,0)+AJ78</f>
         <v/>
       </c>
       <c r="AQ78" s="10" t="n"/>
@@ -11571,7 +11571,7 @@
       </c>
       <c r="B1" s="102" t="inlineStr">
         <is>
-          <t>0.239</t>
+          <t>0.240</t>
         </is>
       </c>
       <c r="C1" s="103" t="inlineStr">
@@ -11581,7 +11581,7 @@
       </c>
       <c r="D1" s="102" t="inlineStr">
         <is>
-          <t>0.239</t>
+          <t>0.240</t>
         </is>
       </c>
       <c r="E1" s="39" t="n"/>

</xml_diff>

<commit_message>
B18: o construir() deixa de parar em Range not found no Sheets — os menus de lista escrita ("a,b,c") vao por requireValueInList no modelo.gs.js, o Ficha.gs e regerado, e o conferir-ficha-xlsx roda o menusSuspensos_ no node contra um Sheets que recusa endereco invalido; e as formulas deixam de dar #ERROR! numa planilha em portugues: o construir() monta em en_US e devolve o idioma num finally; e a ficha montada ganha as bordas dos quatro lados, o formato das caixas vazias e as seis imagens dentro da celula, com o extrair.py guardando o tamanho de tela e o conferir-ficha-xlsx conferindo as tres coisas; e as 47 formulas que citam uma aba criada depois delas passam a ser gravadas numa fila, depois que todas as abas existem; a borda de celula mesclada vai para o bloco inteiro, e as quatro barras (SPARKLINE) saem do embrulho __xludf.DUMMYFUNCTION da exportacao
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ficha-v01/ficha-projeto-m-0.1.xlsx
+++ b/ficha-v01/ficha-projeto-m-0.1.xlsx
@@ -1183,7 +1183,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="15240000" cy="1143000"/>
+    <ext cx="11811000" cy="133350"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -1208,7 +1208,7 @@
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3429000" cy="4381500"/>
+    <ext cx="1809750" cy="2305050"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -1233,7 +1233,7 @@
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="15240000" cy="1143000"/>
+    <ext cx="5334000" cy="104775"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -1258,7 +1258,7 @@
       <row>25</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4000500" cy="4000500"/>
+    <ext cx="1000125" cy="1000125"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -1288,7 +1288,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="15240000" cy="1143000"/>
+    <ext cx="11239500" cy="114300"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -1313,7 +1313,7 @@
       <row>84</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2857500" cy="2857500"/>
+    <ext cx="857250" cy="857250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>

</xml_diff>

<commit_message>
B19 fecha, testado no Sheets; e a ida e volta pelo Sheets fica estavel: a largura de coluna usa a conta do Sheets (pixel = 8 x largura - 1, medida em medidas/larguras-sheets.json), a DADOS deixa de perder a tabela de pericias da coluna AB (o e_da_lista via AB como lista), so entra altura que a planilha declara, texto com cara de numero vai com apostrofo, a aba sem pintura sai sem pintura, e o extrator mantem as imagens que a exportacao traz de dentro da celula
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ficha-v01/ficha-projeto-m-0.1.xlsx
+++ b/ficha-v01/ficha-projeto-m-0.1.xlsx
@@ -11927,7 +11927,11 @@
         </is>
       </c>
       <c r="AA4" s="39" t="n"/>
-      <c r="AB4" s="106" t="n"/>
+      <c r="AB4" s="106" t="inlineStr">
+        <is>
+          <t>perícia</t>
+        </is>
+      </c>
       <c r="AC4" s="106" t="inlineStr">
         <is>
           <t>atributo</t>
@@ -12077,7 +12081,11 @@
         <v>5</v>
       </c>
       <c r="AA5" s="39" t="n"/>
-      <c r="AB5" s="105" t="n"/>
+      <c r="AB5" s="105" t="inlineStr">
+        <is>
+          <t>Atletismo</t>
+        </is>
+      </c>
       <c r="AC5" s="105" t="inlineStr">
         <is>
           <t>Força</t>
@@ -12227,7 +12235,11 @@
         <v>11</v>
       </c>
       <c r="AA6" s="39" t="n"/>
-      <c r="AB6" s="105" t="n"/>
+      <c r="AB6" s="105" t="inlineStr">
+        <is>
+          <t>Acrobacia</t>
+        </is>
+      </c>
       <c r="AC6" s="105" t="inlineStr">
         <is>
           <t>Destreza</t>
@@ -12377,7 +12389,11 @@
         <v>17</v>
       </c>
       <c r="AA7" s="39" t="n"/>
-      <c r="AB7" s="105" t="n"/>
+      <c r="AB7" s="105" t="inlineStr">
+        <is>
+          <t>Furtividade</t>
+        </is>
+      </c>
       <c r="AC7" s="105" t="inlineStr">
         <is>
           <t>Destreza</t>
@@ -12519,7 +12535,11 @@
       </c>
       <c r="Z8" s="39" t="n"/>
       <c r="AA8" s="39" t="n"/>
-      <c r="AB8" s="105" t="n"/>
+      <c r="AB8" s="105" t="inlineStr">
+        <is>
+          <t>Pontaria</t>
+        </is>
+      </c>
       <c r="AC8" s="105" t="inlineStr">
         <is>
           <t>Destreza</t>
@@ -12653,7 +12673,11 @@
       </c>
       <c r="Z9" s="39" t="n"/>
       <c r="AA9" s="39" t="n"/>
-      <c r="AB9" s="105" t="n"/>
+      <c r="AB9" s="105" t="inlineStr">
+        <is>
+          <t>Prestidigitação</t>
+        </is>
+      </c>
       <c r="AC9" s="105" t="inlineStr">
         <is>
           <t>Destreza</t>
@@ -12761,7 +12785,11 @@
       </c>
       <c r="Z10" s="39" t="n"/>
       <c r="AA10" s="39" t="n"/>
-      <c r="AB10" s="105" t="n"/>
+      <c r="AB10" s="105" t="inlineStr">
+        <is>
+          <t>Investigação</t>
+        </is>
+      </c>
       <c r="AC10" s="105" t="inlineStr">
         <is>
           <t>Inteligência</t>
@@ -12865,7 +12893,11 @@
       </c>
       <c r="Z11" s="39" t="n"/>
       <c r="AA11" s="39" t="n"/>
-      <c r="AB11" s="105" t="n"/>
+      <c r="AB11" s="105" t="inlineStr">
+        <is>
+          <t>Intuição</t>
+        </is>
+      </c>
       <c r="AC11" s="105" t="inlineStr">
         <is>
           <t>Inteligência</t>
@@ -12965,7 +12997,11 @@
       <c r="Y12" s="39" t="n"/>
       <c r="Z12" s="39" t="n"/>
       <c r="AA12" s="39" t="n"/>
-      <c r="AB12" s="105" t="n"/>
+      <c r="AB12" s="105" t="inlineStr">
+        <is>
+          <t>Ocultismo</t>
+        </is>
+      </c>
       <c r="AC12" s="105" t="inlineStr">
         <is>
           <t>Inteligência</t>
@@ -13061,7 +13097,11 @@
       <c r="Y13" s="39" t="n"/>
       <c r="Z13" s="39" t="n"/>
       <c r="AA13" s="39" t="n"/>
-      <c r="AB13" s="105" t="n"/>
+      <c r="AB13" s="105" t="inlineStr">
+        <is>
+          <t>Religião</t>
+        </is>
+      </c>
       <c r="AC13" s="105" t="inlineStr">
         <is>
           <t>Inteligência</t>
@@ -13153,7 +13193,11 @@
       <c r="Y14" s="39" t="n"/>
       <c r="Z14" s="39" t="n"/>
       <c r="AA14" s="39" t="n"/>
-      <c r="AB14" s="105" t="n"/>
+      <c r="AB14" s="105" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
       <c r="AC14" s="105" t="inlineStr">
         <is>
           <t>Inteligência</t>
@@ -13241,7 +13285,11 @@
       <c r="Y15" s="39" t="n"/>
       <c r="Z15" s="39" t="n"/>
       <c r="AA15" s="39" t="n"/>
-      <c r="AB15" s="105" t="n"/>
+      <c r="AB15" s="105" t="inlineStr">
+        <is>
+          <t>Hierarquia</t>
+        </is>
+      </c>
       <c r="AC15" s="105" t="inlineStr">
         <is>
           <t>Inteligência</t>
@@ -13329,7 +13377,11 @@
       <c r="Y16" s="39" t="n"/>
       <c r="Z16" s="39" t="n"/>
       <c r="AA16" s="39" t="n"/>
-      <c r="AB16" s="105" t="n"/>
+      <c r="AB16" s="105" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
       <c r="AC16" s="105" t="inlineStr">
         <is>
           <t>Inteligência</t>
@@ -13413,7 +13465,11 @@
       <c r="Y17" s="39" t="n"/>
       <c r="Z17" s="39" t="n"/>
       <c r="AA17" s="39" t="n"/>
-      <c r="AB17" s="105" t="n"/>
+      <c r="AB17" s="105" t="inlineStr">
+        <is>
+          <t>Sobrevivência</t>
+        </is>
+      </c>
       <c r="AC17" s="105" t="inlineStr">
         <is>
           <t>Inteligência</t>
@@ -13497,7 +13553,11 @@
       <c r="Y18" s="39" t="n"/>
       <c r="Z18" s="39" t="n"/>
       <c r="AA18" s="39" t="n"/>
-      <c r="AB18" s="105" t="n"/>
+      <c r="AB18" s="105" t="inlineStr">
+        <is>
+          <t>Natureza</t>
+        </is>
+      </c>
       <c r="AC18" s="105" t="inlineStr">
         <is>
           <t>Inteligência</t>
@@ -13577,7 +13637,11 @@
       <c r="Y19" s="39" t="n"/>
       <c r="Z19" s="39" t="n"/>
       <c r="AA19" s="39" t="n"/>
-      <c r="AB19" s="105" t="n"/>
+      <c r="AB19" s="105" t="inlineStr">
+        <is>
+          <t>Lidar com Animais</t>
+        </is>
+      </c>
       <c r="AC19" s="105" t="inlineStr">
         <is>
           <t>Inteligência</t>
@@ -13657,7 +13721,11 @@
       <c r="Y20" s="39" t="n"/>
       <c r="Z20" s="39" t="n"/>
       <c r="AA20" s="39" t="n"/>
-      <c r="AB20" s="105" t="n"/>
+      <c r="AB20" s="105" t="inlineStr">
+        <is>
+          <t>Tecnologia</t>
+        </is>
+      </c>
       <c r="AC20" s="105" t="inlineStr">
         <is>
           <t>Inteligência</t>
@@ -13737,7 +13805,11 @@
       <c r="Y21" s="39" t="n"/>
       <c r="Z21" s="39" t="n"/>
       <c r="AA21" s="39" t="n"/>
-      <c r="AB21" s="105" t="n"/>
+      <c r="AB21" s="105" t="inlineStr">
+        <is>
+          <t>Sentir Energia</t>
+        </is>
+      </c>
       <c r="AC21" s="105" t="inlineStr">
         <is>
           <t>Essência</t>
@@ -13817,7 +13889,11 @@
       <c r="Y22" s="39" t="n"/>
       <c r="Z22" s="39" t="n"/>
       <c r="AA22" s="39" t="n"/>
-      <c r="AB22" s="105" t="n"/>
+      <c r="AB22" s="105" t="inlineStr">
+        <is>
+          <t>Percepção</t>
+        </is>
+      </c>
       <c r="AC22" s="105" t="inlineStr">
         <is>
           <t>Essência</t>
@@ -13893,7 +13969,11 @@
       <c r="Y23" s="39" t="n"/>
       <c r="Z23" s="39" t="n"/>
       <c r="AA23" s="39" t="n"/>
-      <c r="AB23" s="105" t="n"/>
+      <c r="AB23" s="105" t="inlineStr">
+        <is>
+          <t>Persuasão</t>
+        </is>
+      </c>
       <c r="AC23" s="105" t="inlineStr">
         <is>
           <t>Essência</t>
@@ -13969,7 +14049,11 @@
       <c r="Y24" s="39" t="n"/>
       <c r="Z24" s="39" t="n"/>
       <c r="AA24" s="39" t="n"/>
-      <c r="AB24" s="105" t="n"/>
+      <c r="AB24" s="105" t="inlineStr">
+        <is>
+          <t>Enganação</t>
+        </is>
+      </c>
       <c r="AC24" s="105" t="inlineStr">
         <is>
           <t>Essência</t>
@@ -14045,7 +14129,11 @@
       <c r="Y25" s="39" t="n"/>
       <c r="Z25" s="39" t="n"/>
       <c r="AA25" s="39" t="n"/>
-      <c r="AB25" s="105" t="n"/>
+      <c r="AB25" s="105" t="inlineStr">
+        <is>
+          <t>Intimidação</t>
+        </is>
+      </c>
       <c r="AC25" s="105" t="inlineStr">
         <is>
           <t>Essência</t>
@@ -14121,7 +14209,11 @@
       <c r="Y26" s="39" t="n"/>
       <c r="Z26" s="39" t="n"/>
       <c r="AA26" s="39" t="n"/>
-      <c r="AB26" s="105" t="n"/>
+      <c r="AB26" s="105" t="inlineStr">
+        <is>
+          <t>Atuação</t>
+        </is>
+      </c>
       <c r="AC26" s="105" t="inlineStr">
         <is>
           <t>Essência</t>
@@ -14193,7 +14285,11 @@
       <c r="Y27" s="39" t="n"/>
       <c r="Z27" s="39" t="n"/>
       <c r="AA27" s="39" t="n"/>
-      <c r="AB27" s="105" t="n"/>
+      <c r="AB27" s="105" t="inlineStr">
+        <is>
+          <t>Provocar</t>
+        </is>
+      </c>
       <c r="AC27" s="105" t="inlineStr">
         <is>
           <t>Essência</t>

</xml_diff>

<commit_message>
B3 fecha na opcao A com o refino escolhido: o EQUIPAMENTO vira menu das 27 combinacoes de uniforme e escudo, com a tabela saindo da chave nova equipamento_defesa do catalogo para a DADOS; o REFINO ESCOLHIDO entra ao lado do BLOQUEAR, com o estilo dele, menu, indice e nota; a Defesa corta a Destreza pelo menor teto, a protecao soma o escudo por cima do cobrir-se, e o refino da protecao e do Refino Atual soma as escolhas, uma por marco; o conferir-catalogo confere a chave contra as tabelas do manual, o conferir-ficha-xlsx confere tabela, menus, formulas e notas, e a regressao recalcula dez casos no LibreOffice; o catalogo vai a v0.246
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ficha-v01/ficha-projeto-m-0.1.xlsx
+++ b/ficha-v01/ficha-projeto-m-0.1.xlsx
@@ -5569,16 +5569,20 @@
       <c r="AH36" s="10" t="n"/>
       <c r="AI36" s="11" t="n"/>
       <c r="AJ36" s="46" t="n"/>
-      <c r="AK36" s="46" t="n"/>
-      <c r="AL36" s="46" t="n"/>
-      <c r="AM36" s="46" t="n"/>
-      <c r="AN36" s="46" t="n"/>
-      <c r="AO36" s="46" t="n"/>
-      <c r="AP36" s="46" t="n"/>
-      <c r="AQ36" s="46" t="n"/>
-      <c r="AR36" s="46" t="n"/>
-      <c r="AS36" s="46" t="n"/>
-      <c r="AT36" s="46" t="n"/>
+      <c r="AK36" s="77" t="inlineStr">
+        <is>
+          <t>REFINO ESCOLHIDO</t>
+        </is>
+      </c>
+      <c r="AL36" s="10" t="n"/>
+      <c r="AM36" s="10" t="n"/>
+      <c r="AN36" s="10" t="n"/>
+      <c r="AO36" s="10" t="n"/>
+      <c r="AP36" s="10" t="n"/>
+      <c r="AQ36" s="10" t="n"/>
+      <c r="AR36" s="10" t="n"/>
+      <c r="AS36" s="10" t="n"/>
+      <c r="AT36" s="11" t="n"/>
     </row>
     <row r="37" ht="27" customHeight="1">
       <c r="C37" s="39" t="n"/>
@@ -5624,16 +5628,18 @@
       <c r="AH37" s="10" t="n"/>
       <c r="AI37" s="11" t="n"/>
       <c r="AJ37" s="62" t="n"/>
-      <c r="AK37" s="46" t="n"/>
-      <c r="AL37" s="46" t="n"/>
-      <c r="AM37" s="46" t="n"/>
-      <c r="AN37" s="46" t="n"/>
-      <c r="AO37" s="46" t="n"/>
-      <c r="AP37" s="46" t="n"/>
-      <c r="AQ37" s="46" t="n"/>
-      <c r="AR37" s="46" t="n"/>
-      <c r="AS37" s="46" t="n"/>
-      <c r="AT37" s="46" t="n"/>
+      <c r="AK37" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL37" s="10" t="n"/>
+      <c r="AM37" s="10" t="n"/>
+      <c r="AN37" s="10" t="n"/>
+      <c r="AO37" s="10" t="n"/>
+      <c r="AP37" s="10" t="n"/>
+      <c r="AQ37" s="10" t="n"/>
+      <c r="AR37" s="10" t="n"/>
+      <c r="AS37" s="10" t="n"/>
+      <c r="AT37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="C38" s="39" t="n"/>
@@ -5746,7 +5752,7 @@
     <row r="40" ht="21" customHeight="1">
       <c r="C40" s="39" t="n"/>
       <c r="D40" s="79">
-        <f>10+$L$17+$O$40</f>
+        <f>10+IF($Z$40="",$L$17,MIN($L$17,IFERROR(VALUE(VLOOKUP($Z$40,DADOS!$AE$5:$AH$31,3,FALSE)&amp;""),$L$17)))+$O$40</f>
         <v/>
       </c>
       <c r="E40" s="10" t="n"/>
@@ -5760,7 +5766,7 @@
       <c r="M40" s="11" t="n"/>
       <c r="N40" s="46" t="n"/>
       <c r="O40" s="79">
-        <f>IF($Z$40="",FLOOR((1+COUNTIF(DADOS!$W$5:$W$11,"&lt;="&amp;$AH$11))/3,1)+1,$Z$40)</f>
+        <f>IF($Z$40="",FLOOR(MIN(10,$O$54+MIN($O$54-1,IFERROR(VALUE($AK$37&amp;""),0)))/3,1)+1,IF(VLOOKUP($Z$40,DADOS!$AE$5:$AH$31,4,FALSE)="sim",0,FLOOR(MIN(10,$O$54+MIN($O$54-1,IFERROR(VALUE($AK$37&amp;""),0)))/3,1)+1)+VLOOKUP($Z$40,DADOS!$AE$5:$AH$31,2,FALSE))</f>
         <v/>
       </c>
       <c r="P40" s="10" t="n"/>
@@ -9982,7 +9988,7 @@
       <c r="T116" s="11" t="n"/>
       <c r="U116" s="99" t="n"/>
       <c r="V116" s="97">
-        <f>if(X11 = "Restrição Celestial","Refino ou Lapidação Atual: " &amp; O54+0 &amp; "/10","Refino Atual: " &amp; O54+0 &amp; "/10")</f>
+        <f>if(X11 = "Restrição Celestial","Refino ou Lapidação Atual: " &amp; MIN(10,$O$54+MIN($O$54-1,IFERROR(VALUE($AK$37&amp;""),0))) &amp; "/10","Refino Atual: " &amp; MIN(10,$O$54+MIN($O$54-1,IFERROR(VALUE($AK$37&amp;""),0))) &amp; "/10")</f>
         <v/>
       </c>
       <c r="W116" s="10" t="n"/>
@@ -11130,7 +11136,7 @@
       <c r="AU138" s="39" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="314">
+  <mergeCells count="316">
     <mergeCell ref="P92:Z92"/>
     <mergeCell ref="D2:X2"/>
     <mergeCell ref="D39:M39"/>
@@ -11217,6 +11223,7 @@
     <mergeCell ref="N66:O66"/>
     <mergeCell ref="AF134:AL134"/>
     <mergeCell ref="AB85:AL85"/>
+    <mergeCell ref="AK37:AT37"/>
     <mergeCell ref="AD60:AE60"/>
     <mergeCell ref="N68:O68"/>
     <mergeCell ref="AF23:AK23"/>
@@ -11377,6 +11384,7 @@
     <mergeCell ref="D22:N22"/>
     <mergeCell ref="V64:AC64"/>
     <mergeCell ref="AD69:AE69"/>
+    <mergeCell ref="AK36:AT36"/>
     <mergeCell ref="AF69:AG69"/>
     <mergeCell ref="AM31:AR31"/>
     <mergeCell ref="V136:W136"/>
@@ -11470,7 +11478,7 @@
       <formula>=AND(N(J31)&gt;0,D31/J31&lt;=0.5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="7">
+  <dataValidations count="9">
     <dataValidation sqref="D118:D136" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"0,1,2,3,4,5,6,7,Lib. Max.,Téc. Max."</formula1>
     </dataValidation>
@@ -11491,6 +11499,12 @@
     </dataValidation>
     <dataValidation sqref="X11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>DADOS!$I$4:$I$10</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>DADOS!$AE$5:$AE$31</formula1>
+    </dataValidation>
+    <dataValidation sqref="AK37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"0,1,2,3,4,5,6,7"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11571,7 +11585,7 @@
       </c>
       <c r="B1" s="102" t="inlineStr">
         <is>
-          <t>0.240</t>
+          <t>0.246</t>
         </is>
       </c>
       <c r="C1" s="103" t="inlineStr">
@@ -11581,7 +11595,7 @@
       </c>
       <c r="D1" s="102" t="inlineStr">
         <is>
-          <t>0.240</t>
+          <t>0.246</t>
         </is>
       </c>
       <c r="E1" s="39" t="n"/>
@@ -11938,10 +11952,26 @@
         </is>
       </c>
       <c r="AD4" s="39" t="n"/>
-      <c r="AE4" s="39" t="n"/>
-      <c r="AF4" s="39" t="n"/>
-      <c r="AG4" s="39" t="n"/>
-      <c r="AH4" s="39" t="n"/>
+      <c r="AE4" s="106" t="inlineStr">
+        <is>
+          <t>equipamento</t>
+        </is>
+      </c>
+      <c r="AF4" s="106" t="inlineStr">
+        <is>
+          <t>proteção</t>
+        </is>
+      </c>
+      <c r="AG4" s="106" t="inlineStr">
+        <is>
+          <t>teto de destreza</t>
+        </is>
+      </c>
+      <c r="AH4" s="106" t="inlineStr">
+        <is>
+          <t>desliga a passiva</t>
+        </is>
+      </c>
       <c r="AI4" s="39" t="n"/>
       <c r="AJ4" s="39" t="n"/>
       <c r="AK4" s="39" t="n"/>
@@ -12092,10 +12122,24 @@
         </is>
       </c>
       <c r="AD5" s="39" t="n"/>
-      <c r="AE5" s="39" t="n"/>
-      <c r="AF5" s="39" t="n"/>
-      <c r="AG5" s="39" t="n"/>
-      <c r="AH5" s="39" t="n"/>
+      <c r="AE5" s="105" t="inlineStr">
+        <is>
+          <t>Traje 1</t>
+        </is>
+      </c>
+      <c r="AF5" s="107" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG5" s="107" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH5" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI5" s="39" t="n"/>
       <c r="AJ5" s="39" t="n"/>
       <c r="AK5" s="39" t="n"/>
@@ -12246,10 +12290,24 @@
         </is>
       </c>
       <c r="AD6" s="39" t="n"/>
-      <c r="AE6" s="39" t="n"/>
-      <c r="AF6" s="39" t="n"/>
-      <c r="AG6" s="39" t="n"/>
-      <c r="AH6" s="39" t="n"/>
+      <c r="AE6" s="105" t="inlineStr">
+        <is>
+          <t>Traje 2</t>
+        </is>
+      </c>
+      <c r="AF6" s="107" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG6" s="107" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH6" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI6" s="39" t="n"/>
       <c r="AJ6" s="39" t="n"/>
       <c r="AK6" s="39" t="n"/>
@@ -12400,10 +12458,24 @@
         </is>
       </c>
       <c r="AD7" s="39" t="n"/>
-      <c r="AE7" s="39" t="n"/>
-      <c r="AF7" s="39" t="n"/>
-      <c r="AG7" s="39" t="n"/>
-      <c r="AH7" s="39" t="n"/>
+      <c r="AE7" s="105" t="inlineStr">
+        <is>
+          <t>Traje 3</t>
+        </is>
+      </c>
+      <c r="AF7" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG7" s="107" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH7" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI7" s="39" t="n"/>
       <c r="AJ7" s="39" t="n"/>
       <c r="AK7" s="39" t="n"/>
@@ -12546,10 +12618,22 @@
         </is>
       </c>
       <c r="AD8" s="39" t="n"/>
-      <c r="AE8" s="39" t="n"/>
-      <c r="AF8" s="39" t="n"/>
-      <c r="AG8" s="39" t="n"/>
-      <c r="AH8" s="39" t="n"/>
+      <c r="AE8" s="105" t="inlineStr">
+        <is>
+          <t>Revestimento 1</t>
+        </is>
+      </c>
+      <c r="AF8" s="107" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG8" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI8" s="39" t="n"/>
       <c r="AJ8" s="39" t="n"/>
       <c r="AK8" s="39" t="n"/>
@@ -12684,10 +12768,22 @@
         </is>
       </c>
       <c r="AD9" s="39" t="n"/>
-      <c r="AE9" s="39" t="n"/>
-      <c r="AF9" s="39" t="n"/>
-      <c r="AG9" s="39" t="n"/>
-      <c r="AH9" s="39" t="n"/>
+      <c r="AE9" s="105" t="inlineStr">
+        <is>
+          <t>Revestimento 2</t>
+        </is>
+      </c>
+      <c r="AF9" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG9" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH9" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI9" s="39" t="n"/>
       <c r="AJ9" s="39" t="n"/>
       <c r="AK9" s="39" t="n"/>
@@ -12796,10 +12892,22 @@
         </is>
       </c>
       <c r="AD10" s="39" t="n"/>
-      <c r="AE10" s="39" t="n"/>
-      <c r="AF10" s="39" t="n"/>
-      <c r="AG10" s="39" t="n"/>
-      <c r="AH10" s="39" t="n"/>
+      <c r="AE10" s="105" t="inlineStr">
+        <is>
+          <t>Revestimento 3</t>
+        </is>
+      </c>
+      <c r="AF10" s="107" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG10" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH10" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI10" s="39" t="n"/>
       <c r="AJ10" s="39" t="n"/>
       <c r="AK10" s="39" t="n"/>
@@ -12904,10 +13012,22 @@
         </is>
       </c>
       <c r="AD11" s="39" t="n"/>
-      <c r="AE11" s="39" t="n"/>
-      <c r="AF11" s="39" t="n"/>
-      <c r="AG11" s="39" t="n"/>
-      <c r="AH11" s="39" t="n"/>
+      <c r="AE11" s="105" t="inlineStr">
+        <is>
+          <t>Broquel</t>
+        </is>
+      </c>
+      <c r="AF11" s="107" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG11" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH11" s="107" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="AI11" s="39" t="n"/>
       <c r="AJ11" s="39" t="n"/>
       <c r="AK11" s="39" t="n"/>
@@ -13008,10 +13128,22 @@
         </is>
       </c>
       <c r="AD12" s="39" t="n"/>
-      <c r="AE12" s="39" t="n"/>
-      <c r="AF12" s="39" t="n"/>
-      <c r="AG12" s="39" t="n"/>
-      <c r="AH12" s="39" t="n"/>
+      <c r="AE12" s="105" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="AF12" s="107" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG12" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH12" s="107" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="AI12" s="39" t="n"/>
       <c r="AJ12" s="39" t="n"/>
       <c r="AK12" s="39" t="n"/>
@@ -13108,10 +13240,22 @@
         </is>
       </c>
       <c r="AD13" s="39" t="n"/>
-      <c r="AE13" s="39" t="n"/>
-      <c r="AF13" s="39" t="n"/>
-      <c r="AG13" s="39" t="n"/>
-      <c r="AH13" s="39" t="n"/>
+      <c r="AE13" s="105" t="inlineStr">
+        <is>
+          <t>Torre</t>
+        </is>
+      </c>
+      <c r="AF13" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG13" s="107" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH13" s="107" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="AI13" s="39" t="n"/>
       <c r="AJ13" s="39" t="n"/>
       <c r="AK13" s="39" t="n"/>
@@ -13204,10 +13348,22 @@
         </is>
       </c>
       <c r="AD14" s="39" t="n"/>
-      <c r="AE14" s="39" t="n"/>
-      <c r="AF14" s="39" t="n"/>
-      <c r="AG14" s="39" t="n"/>
-      <c r="AH14" s="39" t="n"/>
+      <c r="AE14" s="105" t="inlineStr">
+        <is>
+          <t>Traje 1 + Broquel</t>
+        </is>
+      </c>
+      <c r="AF14" s="107" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG14" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH14" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI14" s="39" t="n"/>
       <c r="AJ14" s="39" t="n"/>
       <c r="AK14" s="39" t="n"/>
@@ -13296,10 +13452,22 @@
         </is>
       </c>
       <c r="AD15" s="39" t="n"/>
-      <c r="AE15" s="39" t="n"/>
-      <c r="AF15" s="39" t="n"/>
-      <c r="AG15" s="39" t="n"/>
-      <c r="AH15" s="39" t="n"/>
+      <c r="AE15" s="105" t="inlineStr">
+        <is>
+          <t>Traje 1 + Médio</t>
+        </is>
+      </c>
+      <c r="AF15" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG15" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH15" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI15" s="39" t="n"/>
       <c r="AJ15" s="39" t="n"/>
       <c r="AK15" s="39" t="n"/>
@@ -13388,10 +13556,22 @@
         </is>
       </c>
       <c r="AD16" s="39" t="n"/>
-      <c r="AE16" s="39" t="n"/>
-      <c r="AF16" s="39" t="n"/>
-      <c r="AG16" s="39" t="n"/>
-      <c r="AH16" s="39" t="n"/>
+      <c r="AE16" s="105" t="inlineStr">
+        <is>
+          <t>Traje 1 + Torre</t>
+        </is>
+      </c>
+      <c r="AF16" s="107" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG16" s="107" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH16" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI16" s="39" t="n"/>
       <c r="AJ16" s="39" t="n"/>
       <c r="AK16" s="39" t="n"/>
@@ -13476,10 +13656,22 @@
         </is>
       </c>
       <c r="AD17" s="39" t="n"/>
-      <c r="AE17" s="39" t="n"/>
-      <c r="AF17" s="39" t="n"/>
-      <c r="AG17" s="39" t="n"/>
-      <c r="AH17" s="39" t="n"/>
+      <c r="AE17" s="105" t="inlineStr">
+        <is>
+          <t>Traje 2 + Broquel</t>
+        </is>
+      </c>
+      <c r="AF17" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG17" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH17" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI17" s="39" t="n"/>
       <c r="AJ17" s="39" t="n"/>
       <c r="AK17" s="39" t="n"/>
@@ -13564,10 +13756,22 @@
         </is>
       </c>
       <c r="AD18" s="39" t="n"/>
-      <c r="AE18" s="39" t="n"/>
-      <c r="AF18" s="39" t="n"/>
-      <c r="AG18" s="39" t="n"/>
-      <c r="AH18" s="39" t="n"/>
+      <c r="AE18" s="105" t="inlineStr">
+        <is>
+          <t>Traje 2 + Médio</t>
+        </is>
+      </c>
+      <c r="AF18" s="107" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG18" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH18" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI18" s="39" t="n"/>
       <c r="AJ18" s="39" t="n"/>
       <c r="AK18" s="39" t="n"/>
@@ -13648,10 +13852,22 @@
         </is>
       </c>
       <c r="AD19" s="39" t="n"/>
-      <c r="AE19" s="39" t="n"/>
-      <c r="AF19" s="39" t="n"/>
-      <c r="AG19" s="39" t="n"/>
-      <c r="AH19" s="39" t="n"/>
+      <c r="AE19" s="105" t="inlineStr">
+        <is>
+          <t>Traje 2 + Torre</t>
+        </is>
+      </c>
+      <c r="AF19" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG19" s="107" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH19" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI19" s="39" t="n"/>
       <c r="AJ19" s="39" t="n"/>
       <c r="AK19" s="39" t="n"/>
@@ -13732,10 +13948,22 @@
         </is>
       </c>
       <c r="AD20" s="39" t="n"/>
-      <c r="AE20" s="39" t="n"/>
-      <c r="AF20" s="39" t="n"/>
-      <c r="AG20" s="39" t="n"/>
-      <c r="AH20" s="39" t="n"/>
+      <c r="AE20" s="105" t="inlineStr">
+        <is>
+          <t>Traje 3 + Broquel</t>
+        </is>
+      </c>
+      <c r="AF20" s="107" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG20" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH20" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI20" s="39" t="n"/>
       <c r="AJ20" s="39" t="n"/>
       <c r="AK20" s="39" t="n"/>
@@ -13816,10 +14044,22 @@
         </is>
       </c>
       <c r="AD21" s="39" t="n"/>
-      <c r="AE21" s="39" t="n"/>
-      <c r="AF21" s="39" t="n"/>
-      <c r="AG21" s="39" t="n"/>
-      <c r="AH21" s="39" t="n"/>
+      <c r="AE21" s="105" t="inlineStr">
+        <is>
+          <t>Traje 3 + Médio</t>
+        </is>
+      </c>
+      <c r="AF21" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG21" s="107" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH21" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI21" s="39" t="n"/>
       <c r="AJ21" s="39" t="n"/>
       <c r="AK21" s="39" t="n"/>
@@ -13900,10 +14140,22 @@
         </is>
       </c>
       <c r="AD22" s="39" t="n"/>
-      <c r="AE22" s="39" t="n"/>
-      <c r="AF22" s="39" t="n"/>
-      <c r="AG22" s="39" t="n"/>
-      <c r="AH22" s="39" t="n"/>
+      <c r="AE22" s="105" t="inlineStr">
+        <is>
+          <t>Traje 3 + Torre</t>
+        </is>
+      </c>
+      <c r="AF22" s="107" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG22" s="107" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH22" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI22" s="39" t="n"/>
       <c r="AJ22" s="39" t="n"/>
       <c r="AK22" s="39" t="n"/>
@@ -13980,10 +14232,22 @@
         </is>
       </c>
       <c r="AD23" s="39" t="n"/>
-      <c r="AE23" s="39" t="n"/>
-      <c r="AF23" s="39" t="n"/>
-      <c r="AG23" s="39" t="n"/>
-      <c r="AH23" s="39" t="n"/>
+      <c r="AE23" s="105" t="inlineStr">
+        <is>
+          <t>Revestimento 1 + Broquel</t>
+        </is>
+      </c>
+      <c r="AF23" s="107" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG23" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH23" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI23" s="39" t="n"/>
       <c r="AJ23" s="39" t="n"/>
       <c r="AK23" s="39" t="n"/>
@@ -14060,10 +14324,22 @@
         </is>
       </c>
       <c r="AD24" s="39" t="n"/>
-      <c r="AE24" s="39" t="n"/>
-      <c r="AF24" s="39" t="n"/>
-      <c r="AG24" s="39" t="n"/>
-      <c r="AH24" s="39" t="n"/>
+      <c r="AE24" s="105" t="inlineStr">
+        <is>
+          <t>Revestimento 1 + Médio</t>
+        </is>
+      </c>
+      <c r="AF24" s="107" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG24" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH24" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI24" s="39" t="n"/>
       <c r="AJ24" s="39" t="n"/>
       <c r="AK24" s="39" t="n"/>
@@ -14140,10 +14416,22 @@
         </is>
       </c>
       <c r="AD25" s="39" t="n"/>
-      <c r="AE25" s="39" t="n"/>
-      <c r="AF25" s="39" t="n"/>
-      <c r="AG25" s="39" t="n"/>
-      <c r="AH25" s="39" t="n"/>
+      <c r="AE25" s="105" t="inlineStr">
+        <is>
+          <t>Revestimento 1 + Torre</t>
+        </is>
+      </c>
+      <c r="AF25" s="107" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG25" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH25" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI25" s="39" t="n"/>
       <c r="AJ25" s="39" t="n"/>
       <c r="AK25" s="39" t="n"/>
@@ -14220,10 +14508,22 @@
         </is>
       </c>
       <c r="AD26" s="39" t="n"/>
-      <c r="AE26" s="39" t="n"/>
-      <c r="AF26" s="39" t="n"/>
-      <c r="AG26" s="39" t="n"/>
-      <c r="AH26" s="39" t="n"/>
+      <c r="AE26" s="105" t="inlineStr">
+        <is>
+          <t>Revestimento 2 + Broquel</t>
+        </is>
+      </c>
+      <c r="AF26" s="107" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG26" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH26" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI26" s="39" t="n"/>
       <c r="AJ26" s="39" t="n"/>
       <c r="AK26" s="39" t="n"/>
@@ -14296,10 +14596,22 @@
         </is>
       </c>
       <c r="AD27" s="39" t="n"/>
-      <c r="AE27" s="39" t="n"/>
-      <c r="AF27" s="39" t="n"/>
-      <c r="AG27" s="39" t="n"/>
-      <c r="AH27" s="39" t="n"/>
+      <c r="AE27" s="105" t="inlineStr">
+        <is>
+          <t>Revestimento 2 + Médio</t>
+        </is>
+      </c>
+      <c r="AF27" s="107" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG27" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH27" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI27" s="39" t="n"/>
       <c r="AJ27" s="39" t="n"/>
       <c r="AK27" s="39" t="n"/>
@@ -14364,10 +14676,22 @@
       <c r="AB28" s="39" t="n"/>
       <c r="AC28" s="39" t="n"/>
       <c r="AD28" s="39" t="n"/>
-      <c r="AE28" s="39" t="n"/>
-      <c r="AF28" s="39" t="n"/>
-      <c r="AG28" s="39" t="n"/>
-      <c r="AH28" s="39" t="n"/>
+      <c r="AE28" s="105" t="inlineStr">
+        <is>
+          <t>Revestimento 2 + Torre</t>
+        </is>
+      </c>
+      <c r="AF28" s="107" t="n">
+        <v>8</v>
+      </c>
+      <c r="AG28" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH28" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI28" s="39" t="n"/>
       <c r="AJ28" s="39" t="n"/>
       <c r="AK28" s="39" t="n"/>
@@ -14432,10 +14756,22 @@
       <c r="AB29" s="39" t="n"/>
       <c r="AC29" s="39" t="n"/>
       <c r="AD29" s="39" t="n"/>
-      <c r="AE29" s="39" t="n"/>
-      <c r="AF29" s="39" t="n"/>
-      <c r="AG29" s="39" t="n"/>
-      <c r="AH29" s="39" t="n"/>
+      <c r="AE29" s="105" t="inlineStr">
+        <is>
+          <t>Revestimento 3 + Broquel</t>
+        </is>
+      </c>
+      <c r="AF29" s="107" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG29" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH29" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI29" s="39" t="n"/>
       <c r="AJ29" s="39" t="n"/>
       <c r="AK29" s="39" t="n"/>
@@ -14500,10 +14836,22 @@
       <c r="AB30" s="39" t="n"/>
       <c r="AC30" s="39" t="n"/>
       <c r="AD30" s="39" t="n"/>
-      <c r="AE30" s="39" t="n"/>
-      <c r="AF30" s="39" t="n"/>
-      <c r="AG30" s="39" t="n"/>
-      <c r="AH30" s="39" t="n"/>
+      <c r="AE30" s="105" t="inlineStr">
+        <is>
+          <t>Revestimento 3 + Médio</t>
+        </is>
+      </c>
+      <c r="AF30" s="107" t="n">
+        <v>8</v>
+      </c>
+      <c r="AG30" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH30" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI30" s="39" t="n"/>
       <c r="AJ30" s="39" t="n"/>
       <c r="AK30" s="39" t="n"/>
@@ -14568,10 +14916,22 @@
       <c r="AB31" s="39" t="n"/>
       <c r="AC31" s="39" t="n"/>
       <c r="AD31" s="39" t="n"/>
-      <c r="AE31" s="39" t="n"/>
-      <c r="AF31" s="39" t="n"/>
-      <c r="AG31" s="39" t="n"/>
-      <c r="AH31" s="39" t="n"/>
+      <c r="AE31" s="105" t="inlineStr">
+        <is>
+          <t>Revestimento 3 + Torre</t>
+        </is>
+      </c>
+      <c r="AF31" s="107" t="n">
+        <v>9</v>
+      </c>
+      <c r="AG31" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH31" s="107" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="AI31" s="39" t="n"/>
       <c r="AJ31" s="39" t="n"/>
       <c r="AK31" s="39" t="n"/>
@@ -15406,8 +15766,16 @@
       <c r="AX43" s="39" t="n"/>
       <c r="AY43" s="39" t="n"/>
       <c r="AZ43" s="39" t="n"/>
-      <c r="BA43" s="39" t="n"/>
-      <c r="BB43" s="39" t="n"/>
+      <c r="BA43" s="105" t="inlineStr">
+        <is>
+          <t>refino escolhido</t>
+        </is>
+      </c>
+      <c r="BB43" s="105" t="inlineStr">
+        <is>
+          <t>AK37</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="17.25" customHeight="1">
       <c r="A44" s="39" t="n"/>

</xml_diff>